<commit_message>
image start at 0x0800,4000
</commit_message>
<xml_diff>
--- a/ID804/ID804_TEST/Docs/Firmware_Development_Documentation.xlsx
+++ b/ID804/ID804_TEST/Docs/Firmware_Development_Documentation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\ID804\ID804_TEST\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1299E99C-3893-4D8B-922A-B554DA898E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4864B63C-31BC-49DA-8AC4-6346DA338C2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="78660" yWindow="5925" windowWidth="21600" windowHeight="11175" tabRatio="875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" tabRatio="875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirement" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="270">
   <si>
     <t>Requirement ID</t>
   </si>
@@ -920,6 +920,25 @@
   </si>
   <si>
     <t>The The firmware shall support a bootloader.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ARC-009</t>
+  </si>
+  <si>
+    <t>Bootloader</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FW-REQ-007</t>
+  </si>
+  <si>
+    <t>Perform system initialization, firmware image verification, and application jump.
+Support firmware update via UART communication.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>STM32 LL / UART / FLASH</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1023,7 +1042,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1062,9 +1081,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1596,12 +1612,12 @@
     </row>
     <row r="9" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="4" t="s">
-        <v>178</v>
+        <v>267</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="4" t="s">
         <v>264</v>
       </c>
       <c r="E9" s="4" t="s">
@@ -1958,7 +1974,30 @@
       </c>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="11" spans="2:9" ht="34" x14ac:dyDescent="0.45">
+      <c r="B11" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="13"/>
+    </row>
     <row r="13" spans="2:9" ht="17" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <autoFilter ref="B2:I13" xr:uid="{00000000-0009-0000-0000-000001000000}">
@@ -1975,7 +2014,7 @@
           <x14:formula1>
             <xm:f>Common!$D$3:$D$7</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H10</xm:sqref>
+          <xm:sqref>H3:H11</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>